<commit_message>
Angel sheet builder: add Silicon Valley VC and alumni sheets when their data exists
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2WBTUaYVg19XogRfpJJ3d
</commit_message>
<xml_diff>
--- a/collateral/SimReal-天使投资人名单.xlsx
+++ b/collateral/SimReal-天使投资人名单.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'天使名单'!$A$1:$R$92</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'复核未通过'!$A$1:$D$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'复核未通过'!$A$1:$E$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -8970,32 +8970,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>姓名</t>
+          <t>名称</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>现任</t>
+          <t>名单</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>现任 / 地点</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>原因</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>来源</t>
         </is>
@@ -9009,15 +9015,20 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>天使</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>Co-founder, AI Grant / NFDG; founder, Pioneer; joined Meta's new AI lab in 2025</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>投资证据成立。但他2025年7月已加入Meta（SiliconANGLE报道），现在几乎不可能以个人身份投同赛道的初创公司，所以keep=false。</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>https://www.mechanize.work/announcing-mechanize-inc/
 https://finance.yahoo.com/news/mechanize-raises-eyebrows-millions-tech-200252950.html
@@ -9033,15 +9044,20 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>天使</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>Research engineer (pseudonymous), associated with Worldcoin / Tools for Humanity</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>剔除：匿名身份，所在地（含是否在中国大陆）无法核实，无已确认的联系渠道，支票规模可能很小。</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>https://www.theblock.co/post/290476/coinfund-and-distributed-global-lead-5-5-million-seed-round-for-decentralized-ai-firm-prime-intellect
 https://www.coincarp.com/fundraising/prime-intellect-seed/</t>
@@ -9056,15 +9072,20 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
+          <t>天使</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
           <t>Ex-CEO &amp; Chairman, Google</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>投资证据成立。冷邮件几乎触达不到他，而且他不投3周大的公司的小额轮次。keep=false。</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>https://www.maginative.com/article/periodic-labs-launches-with-300m-to-build-an-ai-scientist/
 https://theaiinsider.tech/2025/10/01/periodic-labs-emerges-from-stealth-with-300-million-seed-round-to-build-ai-scientists/
@@ -9080,15 +9101,20 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
+          <t>天使</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
           <t>Co-founder &amp; CEO, Keycard (identity link to the Veris AI angel not confirmed)</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>剔除：Veris融资稿只写“Ian Livingstone”，未写Keycard，存在同名人物（如英国游戏业投资人Sir Ian Livingstone），身份无法确认，有发错人的风险。确认身份后可恢复。</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>https://www.businesswire.com/news/home/20250603868539/en/Veris-AI-Emerges-from-Stealth-with-$8.5M-to-Train-AI-Agents-Using-Simulated-Experience-Removing-Roadblocks-to-Enterprise-Adoption
 https://fintech.global/2025/10/23/keycard-secures-38m-to-advance-ai-agent-security/</t>
@@ -9103,15 +9129,20 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
+          <t>天使</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
           <t>Co-founder, Block; co-founder, Twitter</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>投资证据成立（2024年）。只有一笔AI数据相关投资，可触达性极低，和SimReal的契合度弱。keep=false。</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/mercor-raises-30m-series-a-at-a-250m-valuation-to-create-jobs-with-ai-302252449.html
 https://www.crunchbase.com/funding_round/mercor-dde3-series-a--9ca39ce3
@@ -9127,15 +9158,20 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
+          <t>天使</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
           <t>Professor, Harvard; former US Treasury Secretary</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>投资事实已核实（Mercor Series A名单含Larry Summers），但因声誉风险和淡出公共事务而剔除。</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/mercor-raises-30m-series-a-at-a-250m-valuation-to-create-jobs-with-ai-302252449.html
 https://pulse2.com/mercor-ai-based-hiring-platform-company-closes-30-million-series-a-at-250-million-valuation/</t>
@@ -9150,15 +9186,20 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
+          <t>天使</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
           <t>AI researcher, ex-Google DeepMind / Google Brain (current role not verified)</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>投资事实已核实(2022)，但现职、所在地、联系渠道和近期活跃度全部未知，无法有效触达，剔除。</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/funding_round/perplexity-ai-seed--c8bb7f15
 https://app.dealroom.co/companies/perplexity_ai</t>
@@ -9173,15 +9214,20 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
+          <t>天使</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
           <t>Ex-CEO, GitHub; co-founder, AI Grant / NFDG; reported to have joined Meta's superintelligence effort in 2025</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>投资证据成立。但2025年有报道称他已加入Meta，现在以Meta高管身份投一家同赛道的初创公司可能性很低，所以keep=false。</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>https://www.mechanize.work/announcing-mechanize-inc/
 https://finance.yahoo.com/news/mechanize-raises-eyebrows-millions-tech-200252950.html
@@ -9197,15 +9243,20 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
+          <t>天使</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
           <t>VP of Research &amp; Gemini co-lead, Google DeepMind</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>唯一的公开天使记录是2022年的Perplexity种子轮，太旧了，近两年没有任何记录，所以keep=false。如果能通过剑桥校友找到熟人引荐，可以作为顾问人选另外考虑。</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/funding_round/perplexity-ai-seed--c8bb7f15
 https://synthedia.substack.com/p/perplexity-ai-raises-256-million</t>
@@ -9220,15 +9271,20 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>天使</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>Co-founder, Founders Fund and Palantir; founder, Thiel Fellowship</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>投资证据成立（2024年）。没有公开渠道，冷邮件几乎不可能被读到，日常投资主要通过Founders Fund等机构。keep=false。</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/mercor-raises-30m-series-a-at-a-250m-valuation-to-create-jobs-with-ai-302252449.html
 https://www.crunchbase.com/funding_round/mercor-dde3-series-a--9ca39ce3
@@ -9244,15 +9300,20 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
+          <t>天使</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
           <t>Co-founder &amp; CEO, Carousell</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>剔除：证据陈旧且无年份，赛道完全不相关，无联系渠道。</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>https://vulcanpost.com/724659/carousell-ceo-latest-startup-founder-turned-angel-investor-singapore/
 https://www.crunchbase.com/person/quek-siu-rui</t>
@@ -9267,15 +9328,20 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
+          <t>天使</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
           <t>Not verified (seed data: associated with Nous Research)</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>剔除：单一来源，身份、所在地、现职和联系渠道均无法核实。</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>https://www.theblock.co/post/290476/coinfund-and-distributed-global-lead-5-5-million-seed-round-for-decentralized-ai-firm-prime-intellect</t>
         </is>
@@ -9289,15 +9355,20 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
+          <t>天使</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
           <t>Group Partner, Y Combinator; co-founder, Monzo and GoCardless</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>剔除出天使名单：现为YC合伙人（机构身份），个人天使证据早于加入YC，无2025-2026记录。可作为YC内部的关系人另行联系。Robin AI据报道2025年底陷入困境（本轮未核实），不要在邮件中提。</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>https://sifted.eu/articles/monzo-tom-blomfield-angel-investments
 https://sifted.eu/articles/wise-monzo-founders-generative-ai-news</t>
@@ -9312,15 +9383,20 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
+          <t>天使</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
           <t>Founder, AMI Labs; Professor, NYU; ex-Chief AI Scientist, Meta</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>投资事实已核实(2022)，但无近期天使记录，且技术立场与邮件的LLM-RSI叙事相反，判定不太可能投。原开场白中“improvement measured in P&amp;L”属未经证实的说法，已删除。</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>https://www.crunchbase.com/funding_round/perplexity-ai-seed--c8bb7f15
 https://app.dealroom.co/companies/perplexity_ai</t>
@@ -9335,15 +9411,20 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
+          <t>天使</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
           <t>Co-founder &amp; Executive Chairman, Animoca Brands</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>剔除：没有能确认为个人资金、带年份的天使投资证据，很可能都是Animoca机构出手。香港不属于中国大陆，地域上没问题。</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>https://tracxn.com/d/people/yat-siu/__KRJ9W2iN0CJm23tcIq09Nc_kYAbn-FeEdEiekkSVtFw
 https://signal.nfx.com/investors/yat-siu
@@ -9352,7 +9433,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D16"/>
+  <autoFilter ref="A1:E16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9363,7 +9444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -9372,7 +9453,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>共 91 位个人天使（不含中国大陆）：A 档 15 位，B 档 35 位，C 档 41 位。复核未通过 15 位，单独列出。</t>
+          <t>天使名单：91 位个人天使（不含中国大陆），A 档 15 位，B 档 35 位，C 档 41 位。复核没通过的 15 条单独列在'复核未通过'。</t>
         </is>
       </c>
     </row>
@@ -9413,6 +9494,27 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>硅谷 VC：按首字母逐一列出总部或主要投资团队在旧金山湾区（旧金山、帕洛阿尔托、门洛帕克、山景城等）且 2024–2026 年仍在投的机构，包括种子基金、个人基金、大公司投资部门和投钱的加速器。匹配度：A = 投种子 / 天使轮且投过 AI 基础设施、数据或 agent；B = 早期并投 AI；C = 其他。'已在总表'表示这家也在《非大陆投资人总表》或审批页里。合伙人和投递渠道只列官方公开的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>校友：每位都有来源同时证明他读过剑桥、LSE 或 Duke，并且在做投资；校友天使组织也列在里面。开场句可以提共同的学校。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>大致 / 把握中的条目：部分信息来自调研员已有的知识，没有逐条找到原文，发之前点开官网确认一次。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>导入 Google 表格：drive.google.com → 新建 → 文件上传 → 右键 → 打开方式 → Google 表格。</t>
         </is>

</xml_diff>